<commit_message>
Initialized 27 dash code with display and serial functions, added hall effect sensing capability to 26 T4.1 DAQ code
</commit_message>
<xml_diff>
--- a/PCB/PowerDistributionModule2027/PDM_BOM.xlsx
+++ b/PCB/PowerDistributionModule2027/PDM_BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://svsu0-my.sharepoint.com/personal/wodougla_svsu_edu/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/PowerDistributionModule2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="9" documentId="8_{A4BCC818-4A71-4043-8D32-1B272E8FA4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{396EE566-C633-4F7F-9414-E575FA5FF370}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2562" yWindow="2562" windowWidth="17280" windowHeight="10524" xr2:uid="{71AAA641-6424-472E-9F6E-AB32B794DD02}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{71AAA641-6424-472E-9F6E-AB32B794DD02}"/>
   </bookViews>
   <sheets>
     <sheet name="PDM_BOM" sheetId="2" r:id="rId1"/>
@@ -478,19 +478,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E519D8C-E12F-4CF5-8B72-E44C9C057542}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.20703125" customWidth="1"/>
-    <col min="2" max="2" width="32.1015625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.9453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.3671875" customWidth="1"/>
-    <col min="5" max="5" width="13.5234375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.68359375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.05078125" customWidth="1"/>
-    <col min="8" max="8" width="18.3671875" customWidth="1"/>
+    <col min="1" max="1" width="27.21875" customWidth="1"/>
+    <col min="2" max="2" width="32.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -504,7 +504,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -518,7 +518,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -532,7 +532,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -546,7 +546,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>470</v>
       </c>
@@ -560,7 +560,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>14</v>
       </c>
@@ -573,7 +573,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D944BA0-9763-4063-B197-5C11EB4EE1C1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>